<commit_message>
feat: add nowcasting output indices, figures, and analysis results
</commit_message>
<xml_diff>
--- a/output/nowcasting/impactos_consolidado.xlsx
+++ b/output/nowcasting/impactos_consolidado.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impactos_Consolidados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,190 +441,24 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Impact Total (2026-01-15 -&gt; 2026-01-21)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Impact Total (2026-01-21 -&gt; 2026-02-02)</t>
+          <t>Impact Total (2026-05-26 -&gt; 2026-06-09)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Consumo aparente de cemento - Andalucía</t>
+          <t>Índice general de producción industrial - Andalucía</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>30/11/2025</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1136368599096054</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Consumo aparente de cemento - Andalucía</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>31/10/2025</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0.07654966945184091</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Consumo aparente de cemento - Andalucía</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>31/12/2025</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>-0.02728061210366615</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Matriculación de turismos - Andalucía</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>30/11/2025</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>0.1294959210155535</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Matriculación de turismos - Andalucía</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>31/10/2025</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0.03665626610065128</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Matriculación de turismos - Andalucía</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>31/12/2025</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>-0.07437220551312354</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Ocupados EPA  total - Andalucía</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>31/12/2025</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="n">
-        <v>0.0321614317050364</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Total afiliados SS Total - Andalucía</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>30/11/2025</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0.003198366689348472</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Total afiliados SS Total - Andalucía</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>31/10/2025</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0.008688546201236323</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Total afiliados SS Total - Andalucía</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>31/12/2025</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>-0.006531477311350005</v>
-      </c>
-      <c r="D11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Índice de producción agrícola - Andalucía</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>31/12/2025</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>-0.0004754837074903956</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>0.221542061097848</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>